<commit_message>
Add IFS Functions and update practice file
Add new spreadsheet 'IFS Functions.xlsx' and update the existing 'Basic Practise File.xlsx'. Both are binary Excel file changes; see diff for the file additions and modifications.
</commit_message>
<xml_diff>
--- a/Basic Practise File.xlsx
+++ b/Basic Practise File.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{955ED579-8702-4BB2-8024-54C38A50ACFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11697638-769E-4874-BABF-B3065ABF1C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="955" activeTab="6" xr2:uid="{804A284F-30AB-4AA4-80D9-3863464D9C5B}"/>
   </bookViews>
@@ -1903,7 +1903,7 @@
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C11" s="5">
         <f ca="1">TODAY()</f>
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
   </sheetData>
@@ -2019,7 +2019,7 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <f ca="1">TODAY()</f>
-        <v>46152</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -4068,7 +4068,7 @@
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <f ca="1">RAND()</f>
-        <v>9.8085138375416325E-2</v>
+        <v>0.5022012912003474</v>
       </c>
       <c r="I13" t="s">
         <v>302</v>
@@ -4961,7 +4961,10 @@
       <c r="I3" t="s">
         <v>262</v>
       </c>
-      <c r="J3" s="3"/>
+      <c r="J3" s="3">
+        <f>SUM(G2:G21)</f>
+        <v>184600</v>
+      </c>
       <c r="K3" s="3"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
@@ -4986,7 +4989,10 @@
       <c r="I4" t="s">
         <v>263</v>
       </c>
-      <c r="J4" s="3"/>
+      <c r="J4" s="3">
+        <f>AVERAGE(G2:G21)</f>
+        <v>9230</v>
+      </c>
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
@@ -5014,7 +5020,10 @@
       <c r="I5" t="s">
         <v>264</v>
       </c>
-      <c r="J5" s="3"/>
+      <c r="J5" s="3">
+        <f>MAX(G2:G21)</f>
+        <v>16250</v>
+      </c>
       <c r="K5" s="3"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
@@ -5039,7 +5048,10 @@
       <c r="I6" t="s">
         <v>265</v>
       </c>
-      <c r="J6" s="3"/>
+      <c r="J6" s="3">
+        <f>MIN(G2:G21)</f>
+        <v>4500</v>
+      </c>
       <c r="K6" s="3"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
@@ -5433,7 +5445,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="3">
+  <dataValidations count="3">
     <dataValidation type="custom" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G21" xr:uid="{5536C0C2-2435-420F-96C7-E3A0CA654505}">
       <formula1>ISNUMBER(G2)</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Updated Basic Practise File.xlsx and Mixed Referencing.xlsx
</commit_message>
<xml_diff>
--- a/Basic Practise File.xlsx
+++ b/Basic Practise File.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Besant\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E79BCD-8776-4227-AD27-BA11B573A9D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D6FDCDC-A37F-4875-A373-4966B9CA2DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" tabRatio="955" firstSheet="5" activeTab="10" xr2:uid="{804A284F-30AB-4AA4-80D9-3863464D9C5B}"/>
   </bookViews>
@@ -1153,10 +1153,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -2061,9 +2061,17 @@
       <c r="D2" s="7">
         <v>0.61117256944271503</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="14">
         <f>HOUR(D2)</f>
         <v>14</v>
+      </c>
+      <c r="F2">
+        <f>MINUTE(D2)</f>
+        <v>40</v>
+      </c>
+      <c r="G2">
+        <f>SECOND(D2)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -2073,7 +2081,7 @@
       <c r="B3" t="s">
         <v>174</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="12">
         <v>0.4909722222222222</v>
       </c>
     </row>
@@ -2086,7 +2094,7 @@
       </c>
       <c r="C4" s="5">
         <f ca="1">TODAY()</f>
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="D4" s="5"/>
     </row>
@@ -2099,7 +2107,7 @@
       </c>
       <c r="C5" s="6">
         <f ca="1">NOW()</f>
-        <v>46154.527493171299</v>
+        <v>46155.007678125003</v>
       </c>
       <c r="D5" s="6"/>
     </row>
@@ -2112,7 +2120,7 @@
       </c>
       <c r="C6" s="7">
         <f ca="1">NOW()-TODAY()</f>
-        <v>0.52749317129928386</v>
+        <v>7.678125002712477E-3</v>
       </c>
       <c r="D6" t="s">
         <v>180</v>
@@ -2145,7 +2153,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B9" s="14">
+      <c r="B9">
         <v>1</v>
       </c>
     </row>
@@ -2163,7 +2171,7 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D11" s="5">
         <f ca="1">TODAY()</f>
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
   </sheetData>
@@ -2279,7 +2287,7 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <f ca="1">TODAY()</f>
-        <v>46154</v>
+        <v>46155</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -4328,7 +4336,7 @@
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <f ca="1">RAND()</f>
-        <v>0.14223619048714475</v>
+        <v>0.65154555778481449</v>
       </c>
       <c r="I13" t="s">
         <v>302</v>
@@ -4340,12 +4348,12 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="13" t="s">
         <v>294</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5923,17 +5931,17 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="F3" s="12" t="s">
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="F3" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">

</xml_diff>